<commit_message>
feat: adicionar telas compartilhadas, docs e config EAS Build
Adiciona LgpdConsentScreen, reportHtmlBuilder para exportação de relatórios,
eas.json para builds EAS, checklist de deploy e documentação de funcionalidades.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/HomeCare_Board.xlsx
+++ b/docs/HomeCare_Board.xlsx
@@ -837,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:S78"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="27" min="1" max="1"/>
@@ -860,7 +860,7 @@
     <row r="2" ht="15" customHeight="1" s="28">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>Atualizado em: 14/04/2026 — Estratégia: montar toda a arquitetura de telas e navegação antes de implementar lógica/features</t>
+          <t>Atualizado em: 19/04/2026 — Estratégia: montar toda a arquitetura de telas e navegação antes de implementar lógica/features</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="E35" s="40" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F35" s="38" t="n">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="E36" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F36" s="38" t="n">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="E37" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F37" s="38" t="n">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="E38" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F38" s="38" t="n">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="E39" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F39" s="38" t="n">
@@ -2309,7 +2309,7 @@
       </c>
       <c r="E40" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F40" s="38" t="n">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="E41" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F41" s="38" t="n">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="E42" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F42" s="38" t="n">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="E43" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F43" s="38" t="n">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="E44" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F44" s="38" t="n">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="E45" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F45" s="42" t="n">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="E46" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F46" s="42" t="n">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="E47" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F47" s="42" t="n">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="E48" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F48" s="42" t="n">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="E49" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F49" s="42" t="n">
@@ -2701,7 +2701,7 @@
       </c>
       <c r="E50" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F50" s="42" t="n">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="E51" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F51" s="44" t="n">
@@ -2777,7 +2777,7 @@
       </c>
       <c r="E52" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F52" s="44" t="n">
@@ -2817,7 +2817,7 @@
       </c>
       <c r="E53" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F53" s="44" t="n">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="E54" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F54" s="44" t="n">
@@ -2897,7 +2897,7 @@
       </c>
       <c r="E55" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F55" s="44" t="n">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="E56" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F56" s="44" t="n">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="E57" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F57" s="44" t="n">
@@ -3017,7 +3017,7 @@
       </c>
       <c r="E58" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F58" s="44" t="n">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="E59" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F59" s="46" t="n">
@@ -3089,7 +3089,7 @@
       </c>
       <c r="E60" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F60" s="46" t="n">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="E61" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F61" s="46" t="n">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="E62" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F62" s="46" t="n">
@@ -3197,7 +3197,7 @@
       </c>
       <c r="E63" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F63" s="46" t="n">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="E64" s="41" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F64" s="46" t="n">
@@ -3246,78 +3246,323 @@
       </c>
       <c r="H64" s="47" t="n"/>
     </row>
-    <row r="65"/>
     <row r="66" ht="15" customHeight="1" s="28">
       <c r="A66" s="48" t="inlineStr">
         <is>
-          <t>Resumo</t>
-        </is>
-      </c>
-      <c r="B66" s="48" t="n"/>
+          <t>GEN-75</t>
+        </is>
+      </c>
+      <c r="B66" s="48" t="inlineStr">
+        <is>
+          <t>Fase 6 — Gaps</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>FamilyHomeScreen funcional</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Tela família com dados reais: paciente, registros, plantão</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>3</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Substituiu placeholder por tela completa com Firestore</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="28">
       <c r="A67" s="48" t="inlineStr">
         <is>
-          <t>Total issues:</t>
-        </is>
-      </c>
-      <c r="B67" s="48">
-        <f>COUNTA(A5:A65)</f>
-        <v/>
+          <t>GEN-76</t>
+        </is>
+      </c>
+      <c r="B67" s="48" t="inlineStr">
+        <is>
+          <t>Fase 6 — Gaps</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>ShiftCheckin seleção de paciente</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Checkin com paciente dinâmico (não hardcoded)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>2</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Removido paciente-placeholder, adicionado seletor</t>
+        </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="28">
       <c r="A68" s="48" t="inlineStr">
         <is>
-          <t>Total pontos:</t>
-        </is>
-      </c>
-      <c r="B68" s="48">
-        <f>SUM(F5:F65)</f>
-        <v/>
+          <t>GEN-77</t>
+        </is>
+      </c>
+      <c r="B68" s="48" t="inlineStr">
+        <is>
+          <t>Fase 6 — Gaps</t>
+        </is>
+      </c>
+      <c r="C68" s="27" t="inlineStr">
+        <is>
+          <t>ScheduleScreen + scheduleService Firebase</t>
+        </is>
+      </c>
+      <c r="D68" s="27" t="inlineStr">
+        <is>
+          <t>Escalas lidas do Firestore com mock fallback</t>
+        </is>
+      </c>
+      <c r="E68" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F68" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G68" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H68" s="27" t="inlineStr">
+        <is>
+          <t>scheduleService.ts + integração na tela</t>
+        </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="28">
       <c r="A69" s="48" t="inlineStr">
         <is>
-          <t>Done:</t>
-        </is>
-      </c>
-      <c r="B69" s="48">
-        <f>COUNTIF(E5:E65,"Done")</f>
-        <v/>
+          <t>GEN-78</t>
+        </is>
+      </c>
+      <c r="B69" s="48" t="inlineStr">
+        <is>
+          <t>Fase 6 — Gaps</t>
+        </is>
+      </c>
+      <c r="C69" s="27" t="inlineStr">
+        <is>
+          <t>FinancialScreen + financialService Firebase</t>
+        </is>
+      </c>
+      <c r="D69" s="27" t="inlineStr">
+        <is>
+          <t>Financeiro lido do Firestore com mock fallback</t>
+        </is>
+      </c>
+      <c r="E69" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F69" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G69" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H69" s="27" t="inlineStr">
+        <is>
+          <t>financialService.ts + integração na tela</t>
+        </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="28">
       <c r="A70" s="48" t="inlineStr">
         <is>
-          <t>In Progress:</t>
-        </is>
-      </c>
-      <c r="B70" s="48">
-        <f>COUNTIF(E5:E65,"In Progress")</f>
-        <v/>
+          <t>GEN-79</t>
+        </is>
+      </c>
+      <c r="B70" s="48" t="inlineStr">
+        <is>
+          <t>Fase 6 — Gaps</t>
+        </is>
+      </c>
+      <c r="C70" s="27" t="inlineStr">
+        <is>
+          <t>RegisterPhoto + Firebase Storage upload</t>
+        </is>
+      </c>
+      <c r="D70" s="27" t="inlineStr">
+        <is>
+          <t>Upload de foto vai pro Storage, fallback local</t>
+        </is>
+      </c>
+      <c r="E70" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F70" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G70" s="27" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H70" s="27" t="inlineStr">
+        <is>
+          <t>storageService.ts + integração na tela</t>
+        </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="28">
-      <c r="A71" s="48" t="inlineStr">
-        <is>
-          <t>Blocked:</t>
-        </is>
-      </c>
-      <c r="B71" s="48">
-        <f>COUNTIF(E5:E65,"Blocked")</f>
-        <v/>
-      </c>
+      <c r="A71" s="48" t="n"/>
+      <c r="B71" s="48" t="n"/>
+      <c r="C71" s="27" t="n"/>
+      <c r="D71" s="27" t="n"/>
+      <c r="E71" s="27" t="n"/>
+      <c r="F71" s="27" t="n"/>
+      <c r="G71" s="27" t="n"/>
+      <c r="H71" s="27" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1" s="28">
       <c r="A72" s="48" t="inlineStr">
         <is>
+          <t>Resumo</t>
+        </is>
+      </c>
+      <c r="B72" s="48" t="n"/>
+      <c r="C72" s="27" t="n"/>
+      <c r="D72" s="27" t="n"/>
+      <c r="E72" s="27" t="n"/>
+      <c r="F72" s="27" t="n"/>
+      <c r="G72" s="27" t="n"/>
+      <c r="H72" s="27" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="27" t="inlineStr">
+        <is>
+          <t>Total issues:</t>
+        </is>
+      </c>
+      <c r="B73" s="27">
+        <f>COUNTA(A5:A70)</f>
+        <v/>
+      </c>
+      <c r="C73" s="27" t="n"/>
+      <c r="D73" s="27" t="n"/>
+      <c r="E73" s="27" t="n"/>
+      <c r="F73" s="27" t="n"/>
+      <c r="G73" s="27" t="n"/>
+      <c r="H73" s="27" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="27" t="inlineStr">
+        <is>
+          <t>Total pontos:</t>
+        </is>
+      </c>
+      <c r="B74" s="27">
+        <f>SUM(F5:F70)</f>
+        <v/>
+      </c>
+      <c r="C74" s="27" t="n"/>
+      <c r="D74" s="27" t="n"/>
+      <c r="E74" s="27" t="n"/>
+      <c r="F74" s="27" t="n"/>
+      <c r="G74" s="27" t="n"/>
+      <c r="H74" s="27" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="27" t="inlineStr">
+        <is>
+          <t>Done:</t>
+        </is>
+      </c>
+      <c r="B75" s="27">
+        <f>COUNTIF(E5:E70,"Done")</f>
+        <v/>
+      </c>
+      <c r="C75" s="27" t="n"/>
+      <c r="D75" s="27" t="n"/>
+      <c r="E75" s="27" t="n"/>
+      <c r="F75" s="27" t="n"/>
+      <c r="G75" s="27" t="n"/>
+      <c r="H75" s="27" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="27" t="inlineStr">
+        <is>
+          <t>In Progress:</t>
+        </is>
+      </c>
+      <c r="B76" s="27">
+        <f>COUNTIF(E5:E70,"In Progress")</f>
+        <v/>
+      </c>
+      <c r="C76" s="27" t="n"/>
+      <c r="D76" s="27" t="n"/>
+      <c r="E76" s="27" t="n"/>
+      <c r="F76" s="27" t="n"/>
+      <c r="G76" s="27" t="n"/>
+      <c r="H76" s="27" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="27" t="inlineStr">
+        <is>
+          <t>Blocked:</t>
+        </is>
+      </c>
+      <c r="B77" s="27">
+        <f>COUNTIF(E5:E70,"Blocked")</f>
+        <v/>
+      </c>
+      <c r="C77" s="27" t="n"/>
+      <c r="D77" s="27" t="n"/>
+      <c r="E77" s="27" t="n"/>
+      <c r="F77" s="27" t="n"/>
+      <c r="G77" s="27" t="n"/>
+      <c r="H77" s="27" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="27" t="inlineStr">
+        <is>
           <t>Backlog:</t>
         </is>
       </c>
-      <c r="B72" s="48">
-        <f>COUNTIF(E5:E65,"Backlog")</f>
+      <c r="B78" s="27">
+        <f>COUNTIF(E5:E70,"Backlog")</f>
         <v/>
       </c>
     </row>
@@ -3659,7 +3904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="27" min="1" max="2"/>
@@ -4130,73 +4375,381 @@
       <c r="E20" s="56" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="27" t="inlineStr">
         <is>
           <t>14/04</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="27" t="inlineStr">
         <is>
           <t>GEN-75</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
         <is>
           <t>docs/screens.md com mapa completo de 35 telas</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" s="27" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="27" t="inlineStr">
         <is>
           <t>14/04</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="27" t="inlineStr">
         <is>
           <t>T1-01~20</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
+      <c r="C22" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
         <is>
           <t>25 esqueletos criados + SkeletonScreen + EmptyState</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" s="27" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="27" t="inlineStr">
         <is>
           <t>14/04</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="27" t="inlineStr">
         <is>
           <t>T1-20</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
         <is>
           <t>RootNavigator reescrito: 3 TabNavigators + 10 Stacks</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" s="27" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-14 15:03</t>
+        </is>
+      </c>
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>GEN-61</t>
+        </is>
+      </c>
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>Cadastro de pacientes pelo admin — patientService, CreatePatientScreen, PatientListScreen, AdminPatientDetailScreen implementados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-14 15:33</t>
+        </is>
+      </c>
+      <c r="B25" s="27" t="inlineStr">
+        <is>
+          <t>GEN-46</t>
+        </is>
+      </c>
+      <c r="C25" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
+        <is>
+          <t>NurseHomeScreen (lista pacientes), PatientDetailScreen (info + quick actions), NurseProfileScreen (dados + logout) implementados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-14 15:39</t>
+        </is>
+      </c>
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>GEN-47/48/49</t>
+        </is>
+      </c>
+      <c r="C26" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
+        <is>
+          <t>RegisterMedicationScreen, RegisterVitalsScreen (com alertas fora da faixa), RegisterFeedingScreen + registroService implementados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B27" s="27" t="inlineStr">
+        <is>
+          <t>GEN-50/52/53</t>
+        </is>
+      </c>
+      <c r="C27" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="inlineStr">
+        <is>
+          <t>RegisterActivityScreen, RegisterIncidentScreen, RegisterPhotoScreen implementados. Quick actions do PatientDetailScreen conectados à navegação real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B28" s="27" t="inlineStr">
+        <is>
+          <t>GEN-54</t>
+        </is>
+      </c>
+      <c r="C28" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D28" s="27" t="inlineStr">
+        <is>
+          <t>ShiftEvolutionScreen (SBAR), evolucaoService, QuickRegisterScreen (hub de registros) implementados. Mock patients como fallback em 8 telas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>GEN-55/57/58</t>
+        </is>
+      </c>
+      <c r="C29" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D29" s="27" t="inlineStr">
+        <is>
+          <t>Fase 3 Família: FamilyTimelineScreen (cards por hora, filtra foto clínica), PatientInfoScreen (ficha completa, link gráfico), HistoryFilterScreen (filtro por tipo), FamilyProfileScreen (dados + logout). evolucaoService criado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B30" s="27" t="inlineStr">
+        <is>
+          <t>GEN-59</t>
+        </is>
+      </c>
+      <c r="C30" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D30" s="27" t="inlineStr">
+        <is>
+          <t>VitalsChartScreen: gráficos PA, FC, Temp, SpO₂ (react-native-chart-kit). Seletor de período 7/14/30 dias, mock data fallback, card última aferição, faixas normais do paciente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B31" s="27" t="inlineStr">
+        <is>
+          <t>GEN-60</t>
+        </is>
+      </c>
+      <c r="C31" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D31" s="27" t="inlineStr">
+        <is>
+          <t>ExportReportScreen + reportHtmlBuilder: relatório PDF com seletor de paciente, período (7/14/30/90 dias), filtro por tipo de registro. HTML profissional com header, resumo, tabela de registros. Rota em NurseHomeStack e PatientMgmtStack. Botão "Exportar Relatório PDF" no PatientDetailScreen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B32" s="27" t="inlineStr">
+        <is>
+          <t>GEN-60/62</t>
+        </is>
+      </c>
+      <c r="C32" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D32" s="27" t="inlineStr">
+        <is>
+          <t>ExportReportScreen (PDF com seletor paciente/período/tipo). CreateNurseScreen já implementado (405 linhas). reportHtmlBuilder com HTML profissional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>GEN-63/64/65/66</t>
+        </is>
+      </c>
+      <c r="C33" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D33" s="27" t="inlineStr">
+        <is>
+          <t>Fase 4 Admin completa: LinkFamilyScreen (cria conta família + vincula paciente), AdminDashboardScreen (métricas Firestore: pacientes, profissionais, plantões, registros, intercorrências do dia), TeamListScreen (lista enfermeiros + status), NurseDetailScreen (perfil), ScheduleScreen (grade semanal com turnos), FinancialScreen (receita/despesa/saldo mensal). createFamilyAccount no adminUserService.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B34" s="27" t="inlineStr">
+        <is>
+          <t>GEN-67/68</t>
+        </is>
+      </c>
+      <c r="C34" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D34" s="27" t="inlineStr">
+        <is>
+          <t>GEN-67: Botão "Exportar PDF" na FinancialScreen (HTML profissional com receita/despesa/saldo + tabela lançamentos). GEN-68: Security Rules completas — validação de campos obrigatórios, família não vê fotoClinica, profissionalId == auth.uid nos creates, regra padrão deny-all, soft-delete (status), proteção contra escalação de role.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B35" s="27" t="inlineStr">
+        <is>
+          <t>GEN-67–72</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D35" s="27" t="inlineStr">
+        <is>
+          <t>Fase 5 parcial: GEN-67 export financeiro PDF, GEN-68 security rules completas (LGPD, deny-all, validação campos). GEN-70 LgpdConsentScreen (7 seções, scroll-to-end, salva consentAt no Firestore). GEN-71 auditService (buffer in-memory, preparado para Cloud Functions). GEN-72 tab bar icons (Ionicons) nos 3 perfis. Zero skeletons restantes no projeto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B36" s="27" t="inlineStr">
+        <is>
+          <t>GEN-51/56/73/74</t>
+        </is>
+      </c>
+      <c r="C36" s="27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>GEN-73: app.json completo (permissions iOS/Android, plugins, scheme, EAS config), eas.json (dev/preview/prod profiles, submit config). GEN-51: offlineQueue service (AsyncStorage, auto-retry 30s, max 5 retries, AppState listener, saveRecordWithFallback), useOfflineSync hook, integrado no App.tsx. GEN-56: notificationService (push token registration, Android channels, foreground handler, local scheduling), setupNotificationChannel e handlers no App.tsx. GEN-74: marcado Done (app pronto para teste com usuários).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B37" s="27" t="inlineStr">
+        <is>
+          <t>GEN-56</t>
+        </is>
+      </c>
+      <c r="C37" s="27" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="D37" s="27" t="inlineStr">
+        <is>
+          <t>Push notifications: código pronto (notificationService.ts) mas Blocked — precisa Apple Developer Program pago para testar. Dynamic require garante que não quebra sem o pacote.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:E20"/>

</xml_diff>